<commit_message>
feat(publication): dynamically regenerate Figures 3, 4, 5 and Table 5 from raw alignment data
- Reconcile bSYM to Dx across all models (BioBERT, LLaMA-4, Claude 4.6 Sonnet)
- Update Figure 3 (generate_figure3.py) from raw outputs with class confusions as Conflation (C)
- Update Figure 4 (generate_figure4.py) directly from raw BioBERT seed 42 LOO and LLMs
- Enhance Figure 3 & Figure 4 Overall/Total bar with distinct styling (hatching, divider, shaded background)
- Update Figure 5 (generate_figure5.py): label C as Conflation, revise subtitles 5b & 5c, and reduce word cloud terms to 25
- Update Table 5 (generate_table5.py) to dynamically calculate Leave-One-Out metrics with micro-average aggregation for Total row
- Sync Table 2, Table 5, and Figure artifacts in manuscripts and results
</commit_message>
<xml_diff>
--- a/publication/results/tables/table5_leave_one_out_faers.xlsx
+++ b/publication/results/tables/table5_leave_one_out_faers.xlsx
@@ -18,16 +18,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -38,7 +35,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -46,21 +43,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -426,16 +414,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B7"/>
+  <dimension ref="A1:B8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Metadata Field</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Value</t>
         </is>
@@ -492,24 +480,36 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Evaluation Framework</t>
+          <t>Evaluation Protocol</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>17 Clinical Concept Categories (Two-Tier Evaluation Framework)</t>
+          <t>4-Fold Leave-One-Drug-Event-Pair-Out across 5 Random Seeds (N = 20 Model Runs)</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
+          <t>Aggregation Method</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Micro-Average Aggregated across all 829 reports for total row</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
           <t>Generated By</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>publication/scripts/generate_table5.py</t>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>publication/scripts/generate_table5.py (Computed dynamically from raw.xlsx)</t>
         </is>
       </c>
     </row>
@@ -528,24 +528,24 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Drug–Event Case Series</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Validation Cohort Size</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Strict Exact F1</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>Adapted ADE F1</t>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Primary Tier: Strict Exact F1</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Secondary Tier: Adapted ADE F1</t>
         </is>
       </c>
     </row>
@@ -562,7 +562,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>0.6002 ± 0.0114</t>
+          <t>0.6002 ± 0.0113</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -640,7 +640,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Macro-Average (All 4 Folds)</t>
+          <t>Total (Micro-Average Aggregated)</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -650,12 +650,12 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>0.5685 ± 0.0080</t>
+          <t>0.5564 ± 0.0069</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>0.7463 ± 0.0075</t>
+          <t>0.7420 ± 0.0061</t>
         </is>
       </c>
     </row>

</xml_diff>